<commit_message>
vault sync 2026-10-08 11:17
</commit_message>
<xml_diff>
--- a/2. БИЗНЕС/04_Производство/Активные/2MyMoods/05_Материалы/2026-10-08_Товары_сайта_для_утверждения.xlsx
+++ b/2. БИЗНЕС/04_Производство/Активные/2MyMoods/05_Материалы/2026-10-08_Товары_сайта_для_утверждения.xlsx
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -189,6 +189,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -557,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -623,6 +626,13 @@
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>После ваших отметок заказы переносятся в МойСклад: существующий товар берётся из карточки, новый заводится отдельно, повторных карточек из этой таблицы не создаю.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>8 октября 2026. Все жёлтые строки подтверждены и переведены в существующий товар. Лонгслив из мохера Прочная связь, размер S, артикул 100043, это карточка Лонгслив из мохера "Прочная связь" (сияние) (S). Она лежит в архиве.</t>
         </is>
       </c>
     </row>
@@ -823,2964 +833,3104 @@
       </c>
     </row>
     <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="A2" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы - S</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
         <is>
           <t>100050</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="14" t="inlineStr">
         <is>
           <t>Для склейки не использовал: в старых заказах в артикул часто попадала цена.</t>
         </is>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="I2" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="J2" s="6" t="n">
+      <c r="J2" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="K2" s="7" t="n">
+      <c r="K2" s="17" t="n">
         <v>284185.75</v>
       </c>
-      <c r="L2" s="7" t="n">
+      <c r="L2" s="17" t="n">
         <v>131290.49</v>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="14" t="inlineStr">
         <is>
           <t>2025-12-07</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="14" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="14" t="inlineStr">
         <is>
           <t>В обработке 5, Ошибка оплаты 4, Отменён 1</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="P2" s="14" t="inlineStr">
         <is>
           <t>236012, 236797, 236846, 236847, 236848, 237024, 237025, 237513, 238048, 238736</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="Q2" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R2" s="8" t="inlineStr">
+      <c r="R2" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/plate-s-azhurnymi-vstavkami-ruchnoj-raboty-cherno-belyj/</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr">
+      <c r="S2" s="14" t="inlineStr">
         <is>
           <t>Mon Amour, Все товары</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="T2" s="14" t="inlineStr">
         <is>
           <t>предзаказ</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="U2" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы (черно-белый) (S)</t>
         </is>
       </c>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
-        </is>
-      </c>
-      <c r="Z2" s="4" t="inlineStr">
+      <c r="V2" s="14" t="n"/>
+      <c r="W2" s="14" t="n"/>
+      <c r="X2" s="14" t="n"/>
+      <c r="Y2" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
+        </is>
+      </c>
+      <c r="Z2" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы (черно-белый); Платье-миди с ажурными вставками ручной работы (черно-белый) (M); Платье-миди с ажурными вставками ручной работы (черно-белый) (XS)</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="n"/>
-      <c r="AB2" s="4" t="n"/>
+      <c r="AA2" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB2" s="14" t="n"/>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Платье с вырезом на спине сливочное</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>сливочное</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="6" t="n">
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="K3" s="7" t="n">
+      <c r="K3" s="17" t="n">
         <v>132100</v>
       </c>
-      <c r="L3" s="7" t="n">
+      <c r="L3" s="17" t="n">
         <v>73500</v>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="14" t="inlineStr">
         <is>
           <t>2023-04-27</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" s="14" t="inlineStr">
         <is>
           <t>2023-08-10</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" s="14" t="inlineStr">
         <is>
           <t>Отменён 4, Оплачен 4, Возврат 1</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="P3" s="14" t="inlineStr">
         <is>
           <t>6443, 6490, 6498, 6511, 6534, 6926, 6931, 6975, 7000</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="Q3" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R3" s="4" t="n"/>
-      <c r="S3" s="4" t="n"/>
-      <c r="T3" s="4" t="n"/>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="R3" s="14" t="n"/>
+      <c r="S3" s="14" t="n"/>
+      <c r="T3" s="14" t="n"/>
+      <c r="U3" s="14" t="inlineStr">
         <is>
           <t>Платье с вырезом на спине</t>
         </is>
       </c>
-      <c r="V3" s="4" t="n"/>
-      <c r="W3" s="4" t="n"/>
-      <c r="X3" s="4" t="n"/>
-      <c r="Y3" s="4" t="inlineStr">
-        <is>
-          <t>Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z3" s="4" t="inlineStr">
+      <c r="V3" s="14" t="n"/>
+      <c r="W3" s="14" t="n"/>
+      <c r="X3" s="14" t="n"/>
+      <c r="Y3" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z3" s="14" t="inlineStr">
         <is>
           <t>Платье с вырезом на спине; Платье с вырезом на спине (красный, one size); Платье с вырезом на спине (серый, one size); Платье с вырезом на спине (Оранжевый, one size)</t>
         </is>
       </c>
-      <c r="AA3" s="4" t="n"/>
-      <c r="AB3" s="4" t="n"/>
+      <c r="AA3" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB3" s="14" t="n"/>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы - M</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>100050</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>Для склейки не использовал: в старых заказах в артикул часто попадала цена.</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="J4" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="7" t="n">
+      <c r="K4" s="17" t="n">
         <v>117995.25</v>
       </c>
-      <c r="L4" s="7" t="n">
+      <c r="L4" s="17" t="n">
         <v>68138.10000000001</v>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="14" t="inlineStr">
         <is>
           <t>2025-11-30</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="14" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="O4" s="14" t="inlineStr">
         <is>
           <t>Ошибка оплаты 3, В обработке 1, На удержании 1</t>
         </is>
       </c>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="P4" s="14" t="inlineStr">
         <is>
           <t>235850, 236609, 238666, 238668, 238723</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr">
+      <c r="Q4" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R4" s="8" t="inlineStr">
+      <c r="R4" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/plate-s-azhurnymi-vstavkami-ruchnoj-raboty-cherno-belyj/</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr">
+      <c r="S4" s="14" t="inlineStr">
         <is>
           <t>Mon Amour, Все товары</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
+      <c r="T4" s="14" t="inlineStr">
         <is>
           <t>предзаказ</t>
         </is>
       </c>
-      <c r="U4" s="4" t="inlineStr">
+      <c r="U4" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы (черно-белый) (M)</t>
         </is>
       </c>
-      <c r="V4" s="4" t="n"/>
-      <c r="W4" s="4" t="n"/>
-      <c r="X4" s="4" t="n"/>
-      <c r="Y4" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
-        </is>
-      </c>
-      <c r="Z4" s="4" t="inlineStr">
+      <c r="V4" s="14" t="n"/>
+      <c r="W4" s="14" t="n"/>
+      <c r="X4" s="14" t="n"/>
+      <c r="Y4" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
+        </is>
+      </c>
+      <c r="Z4" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы (черно-белый); Платье-миди с ажурными вставками ручной работы (черно-белый) (S); Платье-миди с ажурными вставками ручной работы (черно-белый) (XS)</t>
         </is>
       </c>
-      <c r="AA4" s="4" t="n"/>
-      <c r="AB4" s="4" t="n"/>
+      <c r="AA4" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB4" s="14" t="n"/>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Кардиган "Care" - Кремовый</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Кремовый</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="6" t="n">
+      <c r="E5" s="14" t="n"/>
+      <c r="F5" s="14" t="n"/>
+      <c r="G5" s="14" t="n"/>
+      <c r="H5" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="K5" s="7" t="n">
+      <c r="K5" s="17" t="n">
         <v>142610</v>
       </c>
-      <c r="L5" s="7" t="n">
+      <c r="L5" s="17" t="n">
         <v>64210</v>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="14" t="inlineStr">
         <is>
           <t>2022-05-12</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N5" s="14" t="inlineStr">
         <is>
           <t>2023-05-21</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="14" t="inlineStr">
         <is>
           <t>Отменён 6, Оплачен 4, Возврат 1</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="P5" s="14" t="inlineStr">
         <is>
           <t>5289, 5290, 5292, 5571, 5572, 5664, 5759, 5792, 5796, 6506, 6585</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="Q5" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R5" s="4" t="n"/>
-      <c r="S5" s="4" t="n"/>
-      <c r="T5" s="4" t="n"/>
-      <c r="U5" s="4" t="inlineStr">
+      <c r="R5" s="14" t="n"/>
+      <c r="S5" s="14" t="n"/>
+      <c r="T5" s="14" t="n"/>
+      <c r="U5" s="14" t="inlineStr">
         <is>
           <t>Кардиган "Care"</t>
         </is>
       </c>
-      <c r="V5" s="4" t="n"/>
-      <c r="W5" s="4" t="n"/>
-      <c r="X5" s="4" t="n"/>
-      <c r="Y5" s="4" t="inlineStr">
-        <is>
-          <t>Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
-        </is>
-      </c>
-      <c r="Z5" s="4" t="inlineStr">
+      <c r="V5" s="14" t="n"/>
+      <c r="W5" s="14" t="n"/>
+      <c r="X5" s="14" t="n"/>
+      <c r="Y5" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
+        </is>
+      </c>
+      <c r="Z5" s="14" t="inlineStr">
         <is>
           <t>Кардиган "Care" (кремовый, S-M); Кардиган "Care" (кремовый, XS)</t>
         </is>
       </c>
-      <c r="AA5" s="4" t="n"/>
-      <c r="AB5" s="4" t="n"/>
+      <c r="AA5" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB5" s="14" t="n"/>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Кардиган с камнями "Облако надежды" - one size</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>one size</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>100003</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>Для склейки не использовал: в старых заказах в артикул часто попадала цена.</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="J6" s="6" t="n">
+      <c r="J6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="K6" s="17" t="n">
         <v>53820</v>
       </c>
-      <c r="L6" s="7" t="n">
+      <c r="L6" s="17" t="n">
         <v>53820</v>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="14" t="inlineStr">
         <is>
           <t>2025-09-13</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" s="14" t="inlineStr">
         <is>
           <t>2025-09-17</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="O6" s="14" t="inlineStr">
         <is>
           <t>В обработке 2</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="P6" s="14" t="inlineStr">
         <is>
           <t>234483, 234551</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="Q6" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R6" s="8" t="inlineStr">
+      <c r="R6" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/kardigan-s-kamnyami-oblako-nadezhdy/</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="S6" s="14" t="inlineStr">
         <is>
           <t>Бестселлеры, Всё по плечу, Все товары, Кардиганы и жакеты, Предзаказ</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="T6" s="14" t="inlineStr">
         <is>
           <t>предзаказ</t>
         </is>
       </c>
-      <c r="U6" s="4" t="inlineStr">
+      <c r="U6" s="14" t="inlineStr">
         <is>
           <t>Кардиган с камнями "Облако надежды" (молочный,  one size)</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr">
+      <c r="V6" s="14" t="inlineStr">
         <is>
           <t>00100003</t>
         </is>
       </c>
-      <c r="W6" s="4" t="inlineStr">
+      <c r="W6" s="14" t="inlineStr">
         <is>
           <t>Жакеты и кардиганы</t>
         </is>
       </c>
-      <c r="X6" s="4" t="n"/>
-      <c r="Y6" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
-        </is>
-      </c>
-      <c r="Z6" s="4" t="n"/>
-      <c r="AA6" s="4" t="n"/>
-      <c r="AB6" s="4" t="n"/>
+      <c r="X6" s="14" t="n"/>
+      <c r="Y6" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
+        </is>
+      </c>
+      <c r="Z6" s="14" t="n"/>
+      <c r="AA6" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB6" s="14" t="n"/>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Кардиган с рукавами-воланами - Бордовый</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Бордовый</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="6" t="n">
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="14" t="n"/>
+      <c r="H7" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="J7" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="K7" s="17" t="n">
         <v>133000</v>
       </c>
-      <c r="L7" s="7" t="n">
+      <c r="L7" s="17" t="n">
         <v>52000</v>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="14" t="inlineStr">
         <is>
           <t>2022-07-31</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="N7" s="14" t="inlineStr">
         <is>
           <t>2023-06-09</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="O7" s="14" t="inlineStr">
         <is>
           <t>Отменён 7, Оплачен 3</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="P7" s="14" t="inlineStr">
         <is>
           <t>5356, 5357, 5358, 5359, 5623, 5773, 5986, 6134, 6486, 6795</t>
         </is>
       </c>
-      <c r="Q7" s="4" t="inlineStr">
+      <c r="Q7" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R7" s="4" t="n"/>
-      <c r="S7" s="4" t="n"/>
-      <c r="T7" s="4" t="n"/>
-      <c r="U7" s="4" t="inlineStr">
+      <c r="R7" s="14" t="n"/>
+      <c r="S7" s="14" t="n"/>
+      <c r="T7" s="14" t="n"/>
+      <c r="U7" s="14" t="inlineStr">
         <is>
           <t>Кардиган с рукавами-воланами</t>
         </is>
       </c>
-      <c r="V7" s="4" t="n"/>
-      <c r="W7" s="4" t="n"/>
-      <c r="X7" s="4" t="n"/>
-      <c r="Y7" s="4" t="inlineStr">
-        <is>
-          <t>Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z7" s="4" t="inlineStr">
+      <c r="V7" s="14" t="n"/>
+      <c r="W7" s="14" t="n"/>
+      <c r="X7" s="14" t="n"/>
+      <c r="Y7" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z7" s="14" t="inlineStr">
         <is>
           <t>Кардиган с рукавами-воланами; Кардиган с рукавами-воланами (черный, one size)</t>
         </is>
       </c>
-      <c r="AA7" s="4" t="n"/>
-      <c r="AB7" s="4" t="n"/>
+      <c r="AA7" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB7" s="14" t="n"/>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Платье "Modest"</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="7" t="n">
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="14" t="n"/>
+      <c r="G8" s="14" t="n"/>
+      <c r="H8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="17" t="n">
         <v>49000</v>
       </c>
-      <c r="L8" s="7" t="n">
+      <c r="L8" s="17" t="n">
         <v>49000</v>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="14" t="inlineStr">
         <is>
           <t>2023-08-10</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="N8" s="14" t="inlineStr">
         <is>
           <t>2023-08-10</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="O8" s="14" t="inlineStr">
         <is>
           <t>Возврат 1</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="P8" s="14" t="inlineStr">
         <is>
           <t>7005</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
+      <c r="Q8" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R8" s="4" t="n"/>
-      <c r="S8" s="4" t="n"/>
-      <c r="T8" s="4" t="n"/>
-      <c r="U8" s="4" t="inlineStr">
+      <c r="R8" s="14" t="n"/>
+      <c r="S8" s="14" t="n"/>
+      <c r="T8" s="14" t="n"/>
+      <c r="U8" s="14" t="inlineStr">
         <is>
           <t>Платье "Modest"</t>
         </is>
       </c>
-      <c r="V8" s="4" t="n"/>
-      <c r="W8" s="4" t="n"/>
-      <c r="X8" s="4" t="n"/>
-      <c r="Y8" s="4" t="inlineStr">
-        <is>
-          <t>Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
-        </is>
-      </c>
-      <c r="Z8" s="4" t="inlineStr">
+      <c r="V8" s="14" t="n"/>
+      <c r="W8" s="14" t="n"/>
+      <c r="X8" s="14" t="n"/>
+      <c r="Y8" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
+        </is>
+      </c>
+      <c r="Z8" s="14" t="inlineStr">
         <is>
           <t>Платье "Modest"; Платье "Modest" (one size, Молочный)</t>
         </is>
       </c>
-      <c r="AA8" s="4" t="n"/>
-      <c r="AB8" s="4" t="n"/>
+      <c r="AA8" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB8" s="14" t="n"/>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Костюм "Мягкое настроение" - серый</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>серый</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>36000</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Похоже на цену, а не на артикул. Для поиска карточки не использовал.</t>
         </is>
       </c>
-      <c r="H9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="7" t="n">
+      <c r="H9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="17" t="n">
         <v>29900</v>
       </c>
-      <c r="L9" s="7" t="n">
+      <c r="L9" s="17" t="n">
         <v>29900</v>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" s="14" t="inlineStr">
         <is>
           <t>2024-01-29</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="N9" s="14" t="inlineStr">
         <is>
           <t>2024-01-29</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="O9" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P9" s="4" t="inlineStr">
+      <c r="P9" s="14" t="inlineStr">
         <is>
           <t>9585</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr">
+      <c r="Q9" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R9" s="8" t="inlineStr">
+      <c r="R9" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/kostyum-myagkoe-nastroenie/</t>
         </is>
       </c>
-      <c r="S9" s="4" t="inlineStr">
+      <c r="S9" s="14" t="inlineStr">
         <is>
           <t>Все товары</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
+      <c r="T9" s="14" t="inlineStr">
         <is>
           <t>предзаказ</t>
         </is>
       </c>
-      <c r="U9" s="4" t="inlineStr">
+      <c r="U9" s="14" t="inlineStr">
         <is>
           <t>Костюм "Мягкое настроение"</t>
         </is>
       </c>
-      <c r="V9" s="4" t="n"/>
-      <c r="W9" s="4" t="n"/>
-      <c r="X9" s="4" t="n"/>
-      <c r="Y9" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z9" s="4" t="inlineStr">
+      <c r="V9" s="14" t="n"/>
+      <c r="W9" s="14" t="n"/>
+      <c r="X9" s="14" t="n"/>
+      <c r="Y9" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z9" s="14" t="inlineStr">
         <is>
           <t>Костюм "Мягкое настроение"; Костюм "Мягкое настроение" (молочный, one size)</t>
         </is>
       </c>
-      <c r="AA9" s="4" t="n"/>
-      <c r="AB9" s="4" t="n"/>
+      <c r="AA9" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB9" s="14" t="n"/>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Кардиган 2MY x Maria Kalashnikova - Графитовый, XS</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Графитовый</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>28000</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>Похоже на цену, а не на артикул. Для поиска карточки не использовал.</t>
         </is>
       </c>
-      <c r="H10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="7" t="n">
+      <c r="H10" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="17" t="n">
         <v>24900</v>
       </c>
-      <c r="L10" s="7" t="n">
+      <c r="L10" s="17" t="n">
         <v>24900</v>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" s="14" t="inlineStr">
         <is>
           <t>2025-01-19</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="N10" s="14" t="inlineStr">
         <is>
           <t>2025-01-19</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="O10" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="P10" s="14" t="inlineStr">
         <is>
           <t>67852</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr">
+      <c r="Q10" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R10" s="8" t="inlineStr">
+      <c r="R10" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/kardigan-2my-x-maria-kalashnikova/</t>
         </is>
       </c>
-      <c r="S10" s="4" t="inlineStr">
+      <c r="S10" s="14" t="inlineStr">
         <is>
           <t>Все товары</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr">
+      <c r="T10" s="14" t="inlineStr">
         <is>
           <t>предзаказ</t>
         </is>
       </c>
-      <c r="U10" s="4" t="inlineStr">
+      <c r="U10" s="14" t="inlineStr">
         <is>
           <t>Кардиган 2MY x Maria Kalashnikova</t>
         </is>
       </c>
-      <c r="V10" s="4" t="n"/>
-      <c r="W10" s="4" t="n"/>
-      <c r="X10" s="4" t="n"/>
-      <c r="Y10" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z10" s="4" t="inlineStr">
+      <c r="V10" s="14" t="n"/>
+      <c r="W10" s="14" t="n"/>
+      <c r="X10" s="14" t="n"/>
+      <c r="Y10" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z10" s="14" t="inlineStr">
         <is>
           <t>Кардиган 2MY x Maria Kalashnikova; Кардиган 2MY x Maria Kalashnikova (Молочный, S-M); Кардиган 2MY x Maria Kalashnikova (Молочный, XS); Кардиган 2MY x Maria Kalashnikova (XS, Шоколадный); Кардиган 2MY x Maria Kalashnikova (S-M, Шоколадный)</t>
         </is>
       </c>
-      <c r="AA10" s="4" t="n"/>
-      <c r="AB10" s="4" t="n"/>
+      <c r="AA10" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB10" s="14" t="n"/>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Платье Bloom</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="6" t="n">
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
+      <c r="G11" s="14" t="n"/>
+      <c r="H11" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="6" t="n">
+      <c r="I11" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="K11" s="7" t="n">
+      <c r="K11" s="17" t="n">
         <v>65700</v>
       </c>
-      <c r="L11" s="7" t="n">
+      <c r="L11" s="17" t="n">
         <v>21900</v>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" s="14" t="inlineStr">
         <is>
           <t>2023-05-23</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="N11" s="14" t="inlineStr">
         <is>
           <t>2023-07-05</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="O11" s="14" t="inlineStr">
         <is>
           <t>Отменён 2, Оплачен 1</t>
         </is>
       </c>
-      <c r="P11" s="4" t="inlineStr">
+      <c r="P11" s="14" t="inlineStr">
         <is>
           <t>6589, 6716, 6928</t>
         </is>
       </c>
-      <c r="Q11" s="4" t="inlineStr">
+      <c r="Q11" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R11" s="4" t="n"/>
-      <c r="S11" s="4" t="n"/>
-      <c r="T11" s="4" t="n"/>
-      <c r="U11" s="4" t="inlineStr">
+      <c r="R11" s="14" t="n"/>
+      <c r="S11" s="14" t="n"/>
+      <c r="T11" s="14" t="n"/>
+      <c r="U11" s="14" t="inlineStr">
         <is>
           <t>Платье "Bloom"</t>
         </is>
       </c>
-      <c r="V11" s="4" t="n"/>
-      <c r="W11" s="4" t="n"/>
-      <c r="X11" s="4" t="n"/>
-      <c r="Y11" s="4" t="inlineStr">
-        <is>
-          <t>Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
-        </is>
-      </c>
-      <c r="Z11" s="4" t="inlineStr">
+      <c r="V11" s="14" t="n"/>
+      <c r="W11" s="14" t="n"/>
+      <c r="X11" s="14" t="n"/>
+      <c r="Y11" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
+        </is>
+      </c>
+      <c r="Z11" s="14" t="inlineStr">
         <is>
           <t>Платье "Bloom"; Платье "Bloom" (лимонный, one size); Платье "Bloom" (черный, one size)</t>
         </is>
       </c>
-      <c r="AA11" s="4" t="n"/>
-      <c r="AB11" s="4" t="n"/>
+      <c r="AA11" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB11" s="14" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы - XS</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>100050</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>Для склейки не использовал: в старых заказах в артикул часто попадала цена.</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="7" t="n">
+      <c r="H12" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="17" t="n">
         <v>16619.05</v>
       </c>
-      <c r="L12" s="7" t="n">
+      <c r="L12" s="17" t="n">
         <v>16619.05</v>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M12" s="14" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N12" s="14" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="O12" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="P12" s="14" t="inlineStr">
         <is>
           <t>238696</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
+      <c r="Q12" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R12" s="8" t="inlineStr">
+      <c r="R12" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/plate-s-azhurnymi-vstavkami-ruchnoj-raboty-cherno-belyj/</t>
         </is>
       </c>
-      <c r="S12" s="4" t="inlineStr">
+      <c r="S12" s="14" t="inlineStr">
         <is>
           <t>Mon Amour, Все товары</t>
         </is>
       </c>
-      <c r="T12" s="4" t="n"/>
-      <c r="U12" s="4" t="inlineStr">
+      <c r="T12" s="14" t="n"/>
+      <c r="U12" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы (черно-белый) (XS)</t>
         </is>
       </c>
-      <c r="V12" s="4" t="n"/>
-      <c r="W12" s="4" t="n"/>
-      <c r="X12" s="4" t="n"/>
-      <c r="Y12" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
-        </is>
-      </c>
-      <c r="Z12" s="4" t="inlineStr">
+      <c r="V12" s="14" t="n"/>
+      <c r="W12" s="14" t="n"/>
+      <c r="X12" s="14" t="n"/>
+      <c r="Y12" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
+        </is>
+      </c>
+      <c r="Z12" s="14" t="inlineStr">
         <is>
           <t>Платье-миди с ажурными вставками ручной работы (черно-белый); Платье-миди с ажурными вставками ручной работы (черно-белый) (M); Платье-миди с ажурными вставками ручной работы (черно-белый) (S)</t>
         </is>
       </c>
-      <c r="AA12" s="4" t="n"/>
-      <c r="AB12" s="4" t="n"/>
+      <c r="AA12" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB12" s="14" t="n"/>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>Подарочный сертификат 2mymoods - 20000</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>20000</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="7" t="n">
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n"/>
+      <c r="G13" s="14" t="n"/>
+      <c r="H13" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="17" t="n">
         <v>15000</v>
       </c>
-      <c r="L13" s="7" t="n">
+      <c r="L13" s="17" t="n">
         <v>15000</v>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="M13" s="14" t="inlineStr">
         <is>
           <t>2023-04-17</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="N13" s="14" t="inlineStr">
         <is>
           <t>2023-04-17</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="O13" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P13" s="4" t="inlineStr">
+      <c r="P13" s="14" t="inlineStr">
         <is>
           <t>6386</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="Q13" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R13" s="4" t="n"/>
-      <c r="S13" s="4" t="n"/>
-      <c r="T13" s="4" t="inlineStr">
+      <c r="R13" s="14" t="n"/>
+      <c r="S13" s="14" t="n"/>
+      <c r="T13" s="14" t="inlineStr">
         <is>
           <t>сертификат на 20000</t>
         </is>
       </c>
-      <c r="U13" s="4" t="inlineStr">
+      <c r="U13" s="14" t="inlineStr">
         <is>
           <t>Подарочный сертификат (20000)</t>
         </is>
       </c>
-      <c r="V13" s="4" t="n"/>
-      <c r="W13" s="4" t="n"/>
-      <c r="X13" s="4" t="n"/>
-      <c r="Y13" s="4" t="inlineStr">
-        <is>
-          <t>Номинал сертификата совпал с карточкой склада.</t>
-        </is>
-      </c>
-      <c r="Z13" s="4" t="inlineStr">
+      <c r="V13" s="14" t="n"/>
+      <c r="W13" s="14" t="n"/>
+      <c r="X13" s="14" t="n"/>
+      <c r="Y13" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Номинал сертификата совпал с карточкой склада.</t>
+        </is>
+      </c>
+      <c r="Z13" s="14" t="inlineStr">
         <is>
           <t>Подарочный сертификат; Подарочный сертификат (10000); Подарочный сертификат (15000); Подарочный сертификат (5000); Подарочный сертификат</t>
         </is>
       </c>
-      <c r="AA13" s="4" t="n"/>
-      <c r="AB13" s="4" t="n"/>
+      <c r="AA13" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB13" s="14" t="n"/>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Жилет с горлом - S-M</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>S-M</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>27000</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>Похоже на цену, а не на артикул. Для поиска карточки не использовал.</t>
         </is>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="J14" s="6" t="n">
+      <c r="J14" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="7" t="n">
+      <c r="K14" s="17" t="n">
         <v>14850</v>
       </c>
-      <c r="L14" s="7" t="n">
+      <c r="L14" s="17" t="n">
         <v>14850</v>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M14" s="14" t="inlineStr">
         <is>
           <t>2024-11-01</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N14" s="14" t="inlineStr">
         <is>
           <t>2025-03-15</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="O14" s="14" t="inlineStr">
         <is>
           <t>В обработке 1, Оплачен 1</t>
         </is>
       </c>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="P14" s="14" t="inlineStr">
         <is>
           <t>13625, 158152</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="Q14" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R14" s="8" t="inlineStr">
+      <c r="R14" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/?post_type=product&amp;p=12949</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
+      <c r="S14" s="14" t="inlineStr">
         <is>
           <t>Все товары</t>
         </is>
       </c>
-      <c r="T14" s="4" t="n"/>
-      <c r="U14" s="4" t="inlineStr">
+      <c r="T14" s="14" t="n"/>
+      <c r="U14" s="14" t="inlineStr">
         <is>
           <t>Жилет с горлом (Розовый, S-M)</t>
         </is>
       </c>
-      <c r="V14" s="4" t="n"/>
-      <c r="W14" s="4" t="n"/>
-      <c r="X14" s="4" t="n"/>
-      <c r="Y14" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
-        </is>
-      </c>
-      <c r="Z14" s="4" t="inlineStr">
+      <c r="V14" s="14" t="n"/>
+      <c r="W14" s="14" t="n"/>
+      <c r="X14" s="14" t="n"/>
+      <c r="Y14" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. В заказе указан размер, цвет не указан. В этом размере на складе одна карточка, проверьте цвет.</t>
+        </is>
+      </c>
+      <c r="Z14" s="14" t="inlineStr">
         <is>
           <t>Жилет с горлом</t>
         </is>
       </c>
-      <c r="AA14" s="4" t="n"/>
-      <c r="AB14" s="4" t="n"/>
+      <c r="AA14" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB14" s="14" t="n"/>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Кардиган "Care" - Молочно-бежевый</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Молочно-бежевый</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
-      <c r="H15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="7" t="n">
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n"/>
+      <c r="G15" s="14" t="n"/>
+      <c r="H15" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="17" t="n">
         <v>12900</v>
       </c>
-      <c r="L15" s="7" t="n">
+      <c r="L15" s="17" t="n">
         <v>12900</v>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M15" s="14" t="inlineStr">
         <is>
           <t>2022-09-01</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="N15" s="14" t="inlineStr">
         <is>
           <t>2022-09-01</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr">
+      <c r="O15" s="14" t="inlineStr">
         <is>
           <t>Возврат 1</t>
         </is>
       </c>
-      <c r="P15" s="4" t="inlineStr">
+      <c r="P15" s="14" t="inlineStr">
         <is>
           <t>5418</t>
         </is>
       </c>
-      <c r="Q15" s="4" t="inlineStr">
+      <c r="Q15" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R15" s="4" t="n"/>
-      <c r="S15" s="4" t="n"/>
-      <c r="T15" s="4" t="n"/>
-      <c r="U15" s="4" t="inlineStr">
+      <c r="R15" s="14" t="n"/>
+      <c r="S15" s="14" t="n"/>
+      <c r="T15" s="14" t="n"/>
+      <c r="U15" s="14" t="inlineStr">
         <is>
           <t>Кардиган "Care"</t>
         </is>
       </c>
-      <c r="V15" s="4" t="n"/>
-      <c r="W15" s="4" t="n"/>
-      <c r="X15" s="4" t="n"/>
-      <c r="Y15" s="4" t="inlineStr">
-        <is>
-          <t>Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z15" s="4" t="inlineStr">
+      <c r="V15" s="14" t="n"/>
+      <c r="W15" s="14" t="n"/>
+      <c r="X15" s="14" t="n"/>
+      <c r="Y15" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z15" s="14" t="inlineStr">
         <is>
           <t>Кардиган "Care"; Кардиган "Care" (кремовый, S-M); Кардиган "Care" (кремовый, XS)</t>
         </is>
       </c>
-      <c r="AA15" s="4" t="n"/>
-      <c r="AB15" s="4" t="n"/>
+      <c r="AA15" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB15" s="14" t="n"/>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Юбка макси черная</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>черная</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="7" t="n">
+      <c r="E16" s="14" t="n"/>
+      <c r="F16" s="14" t="n"/>
+      <c r="G16" s="14" t="n"/>
+      <c r="H16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="17" t="n">
         <v>11900</v>
       </c>
-      <c r="L16" s="7" t="n">
+      <c r="L16" s="17" t="n">
         <v>11900</v>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M16" s="14" t="inlineStr">
         <is>
           <t>2023-09-07</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="N16" s="14" t="inlineStr">
         <is>
           <t>2023-09-07</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="O16" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P16" s="4" t="inlineStr">
+      <c r="P16" s="14" t="inlineStr">
         <is>
           <t>7250</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr">
+      <c r="Q16" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R16" s="4" t="n"/>
-      <c r="S16" s="4" t="n"/>
-      <c r="T16" s="4" t="n"/>
-      <c r="U16" s="4" t="inlineStr">
+      <c r="R16" s="14" t="n"/>
+      <c r="S16" s="14" t="n"/>
+      <c r="T16" s="14" t="n"/>
+      <c r="U16" s="14" t="inlineStr">
         <is>
           <t>Юбка макси</t>
         </is>
       </c>
-      <c r="V16" s="4" t="n"/>
-      <c r="W16" s="4" t="n"/>
-      <c r="X16" s="4" t="n"/>
-      <c r="Y16" s="4" t="inlineStr">
-        <is>
-          <t>Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
-        </is>
-      </c>
-      <c r="Z16" s="4" t="inlineStr">
+      <c r="V16" s="14" t="n"/>
+      <c r="W16" s="14" t="n"/>
+      <c r="X16" s="14" t="n"/>
+      <c r="Y16" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
+        </is>
+      </c>
+      <c r="Z16" s="14" t="inlineStr">
         <is>
           <t>Юбка макси (Черный, S-M); Юбка макси (Черный, XS)</t>
         </is>
       </c>
-      <c r="AA16" s="4" t="n"/>
-      <c r="AB16" s="4" t="n"/>
+      <c r="AA16" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB16" s="14" t="n"/>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Чепчик "Звездное небо" - серый</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>серый</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="7" t="n">
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="17" t="n">
         <v>7900</v>
       </c>
-      <c r="L17" s="7" t="n">
+      <c r="L17" s="17" t="n">
         <v>7900</v>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="M17" s="14" t="inlineStr">
         <is>
           <t>2024-01-29</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="N17" s="14" t="inlineStr">
         <is>
           <t>2024-01-29</t>
         </is>
       </c>
-      <c r="O17" s="4" t="inlineStr">
+      <c r="O17" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P17" s="4" t="inlineStr">
+      <c r="P17" s="14" t="inlineStr">
         <is>
           <t>9586</t>
         </is>
       </c>
-      <c r="Q17" s="4" t="inlineStr">
+      <c r="Q17" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R17" s="4" t="n"/>
-      <c r="S17" s="4" t="n"/>
-      <c r="T17" s="4" t="inlineStr">
+      <c r="R17" s="14" t="n"/>
+      <c r="S17" s="14" t="n"/>
+      <c r="T17" s="14" t="inlineStr">
         <is>
           <t>предзаказ</t>
         </is>
       </c>
-      <c r="U17" s="4" t="inlineStr">
+      <c r="U17" s="14" t="inlineStr">
         <is>
           <t>Чепчик "Звездное небо"</t>
         </is>
       </c>
-      <c r="V17" s="4" t="n"/>
-      <c r="W17" s="4" t="n"/>
-      <c r="X17" s="4" t="n"/>
-      <c r="Y17" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z17" s="4" t="inlineStr">
+      <c r="V17" s="14" t="n"/>
+      <c r="W17" s="14" t="n"/>
+      <c r="X17" s="14" t="n"/>
+      <c r="Y17" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z17" s="14" t="inlineStr">
         <is>
           <t>Чепчик "Звездное небо"; Чепчик "Звездное небо" (белый, one size)</t>
         </is>
       </c>
-      <c r="AA17" s="4" t="n"/>
-      <c r="AB17" s="4" t="n"/>
+      <c r="AA17" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB17" s="14" t="n"/>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Манжеты - Черный</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Черный</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="6" t="n">
+      <c r="E18" s="14" t="n"/>
+      <c r="F18" s="14" t="n"/>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="6" t="n">
+      <c r="I18" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="K18" s="7" t="n">
+      <c r="K18" s="17" t="n">
         <v>11700</v>
       </c>
-      <c r="L18" s="7" t="n">
+      <c r="L18" s="17" t="n">
         <v>3900</v>
       </c>
-      <c r="M18" s="4" t="inlineStr">
+      <c r="M18" s="14" t="inlineStr">
         <is>
           <t>2023-05-16</t>
         </is>
       </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="N18" s="14" t="inlineStr">
         <is>
           <t>2023-08-30</t>
         </is>
       </c>
-      <c r="O18" s="4" t="inlineStr">
+      <c r="O18" s="14" t="inlineStr">
         <is>
           <t>Отменён 2, Оплачен 1</t>
         </is>
       </c>
-      <c r="P18" s="4" t="inlineStr">
+      <c r="P18" s="14" t="inlineStr">
         <is>
           <t>6536, 6887, 7202</t>
         </is>
       </c>
-      <c r="Q18" s="4" t="inlineStr">
+      <c r="Q18" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R18" s="4" t="n"/>
-      <c r="S18" s="4" t="n"/>
-      <c r="T18" s="4" t="n"/>
-      <c r="U18" s="4" t="inlineStr">
+      <c r="R18" s="14" t="n"/>
+      <c r="S18" s="14" t="n"/>
+      <c r="T18" s="14" t="n"/>
+      <c r="U18" s="14" t="inlineStr">
         <is>
           <t>Манжеты (черный, one size)</t>
         </is>
       </c>
-      <c r="V18" s="4" t="n"/>
-      <c r="W18" s="4" t="n"/>
-      <c r="X18" s="4" t="n"/>
-      <c r="Y18" s="4" t="inlineStr">
-        <is>
-          <t>Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
-        </is>
-      </c>
-      <c r="Z18" s="4" t="n"/>
-      <c r="AA18" s="4" t="n"/>
-      <c r="AB18" s="4" t="n"/>
+      <c r="V18" s="14" t="n"/>
+      <c r="W18" s="14" t="n"/>
+      <c r="X18" s="14" t="n"/>
+      <c r="Y18" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
+        </is>
+      </c>
+      <c r="Z18" s="14" t="n"/>
+      <c r="AA18" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB18" s="14" t="n"/>
     </row>
     <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>Манжеты - Сливочный</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>Сливочный</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="7" t="n">
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="17" t="n">
         <v>3900</v>
       </c>
-      <c r="L19" s="7" t="n">
+      <c r="L19" s="17" t="n">
         <v>3900</v>
       </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="M19" s="14" t="inlineStr">
         <is>
           <t>2023-04-12</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="N19" s="14" t="inlineStr">
         <is>
           <t>2023-04-12</t>
         </is>
       </c>
-      <c r="O19" s="4" t="inlineStr">
+      <c r="O19" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P19" s="4" t="inlineStr">
+      <c r="P19" s="14" t="inlineStr">
         <is>
           <t>6295</t>
         </is>
       </c>
-      <c r="Q19" s="4" t="inlineStr">
+      <c r="Q19" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R19" s="4" t="n"/>
-      <c r="S19" s="4" t="n"/>
-      <c r="T19" s="4" t="n"/>
-      <c r="U19" s="4" t="inlineStr">
+      <c r="R19" s="14" t="n"/>
+      <c r="S19" s="14" t="n"/>
+      <c r="T19" s="14" t="n"/>
+      <c r="U19" s="14" t="inlineStr">
         <is>
           <t>Манжеты (сливочный, one size)</t>
         </is>
       </c>
-      <c r="V19" s="4" t="n"/>
-      <c r="W19" s="4" t="n"/>
-      <c r="X19" s="4" t="n"/>
-      <c r="Y19" s="4" t="inlineStr">
-        <is>
-          <t>Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
-        </is>
-      </c>
-      <c r="Z19" s="4" t="n"/>
-      <c r="AA19" s="4" t="n"/>
-      <c r="AB19" s="4" t="n"/>
+      <c r="V19" s="14" t="n"/>
+      <c r="W19" s="14" t="n"/>
+      <c r="X19" s="14" t="n"/>
+      <c r="Y19" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
+        </is>
+      </c>
+      <c r="Z19" s="14" t="n"/>
+      <c r="AA19" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB19" s="14" t="n"/>
     </row>
     <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Топ "Touch" - Кремовый</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Кремовый</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="7" t="n">
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="14" t="n"/>
+      <c r="G20" s="14" t="n"/>
+      <c r="H20" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="17" t="n">
         <v>3900</v>
       </c>
-      <c r="L20" s="7" t="n">
+      <c r="L20" s="17" t="n">
         <v>3900</v>
       </c>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="M20" s="14" t="inlineStr">
         <is>
           <t>2023-05-11</t>
         </is>
       </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="N20" s="14" t="inlineStr">
         <is>
           <t>2023-05-11</t>
         </is>
       </c>
-      <c r="O20" s="4" t="inlineStr">
+      <c r="O20" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P20" s="4" t="inlineStr">
+      <c r="P20" s="14" t="inlineStr">
         <is>
           <t>6505</t>
         </is>
       </c>
-      <c r="Q20" s="4" t="inlineStr">
+      <c r="Q20" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R20" s="4" t="n"/>
-      <c r="S20" s="4" t="n"/>
-      <c r="T20" s="4" t="n"/>
-      <c r="U20" s="4" t="inlineStr">
+      <c r="R20" s="14" t="n"/>
+      <c r="S20" s="14" t="n"/>
+      <c r="T20" s="14" t="n"/>
+      <c r="U20" s="14" t="inlineStr">
         <is>
           <t>Топ "Touch" (кремовый, one size)</t>
         </is>
       </c>
-      <c r="V20" s="4" t="n"/>
-      <c r="W20" s="4" t="n"/>
-      <c r="X20" s="4" t="n"/>
-      <c r="Y20" s="4" t="inlineStr">
-        <is>
-          <t>Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
-        </is>
-      </c>
-      <c r="Z20" s="4" t="n"/>
-      <c r="AA20" s="4" t="n"/>
-      <c r="AB20" s="4" t="n"/>
+      <c r="V20" s="14" t="n"/>
+      <c r="W20" s="14" t="n"/>
+      <c r="X20" s="14" t="n"/>
+      <c r="Y20" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
+        </is>
+      </c>
+      <c r="Z20" s="14" t="n"/>
+      <c r="AA20" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB20" s="14" t="n"/>
     </row>
     <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" - Бледно-розовый</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>Бледно-розовый</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
-      <c r="H21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="7" t="n">
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="L21" s="7" t="n">
+      <c r="L21" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="M21" s="14" t="inlineStr">
         <is>
           <t>2023-04-25</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="N21" s="14" t="inlineStr">
         <is>
           <t>2023-04-25</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr">
+      <c r="O21" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P21" s="4" t="inlineStr">
+      <c r="P21" s="14" t="inlineStr">
         <is>
           <t>6411</t>
         </is>
       </c>
-      <c r="Q21" s="4" t="inlineStr">
+      <c r="Q21" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R21" s="4" t="n"/>
-      <c r="S21" s="4" t="n"/>
-      <c r="T21" s="4" t="n"/>
-      <c r="U21" s="4" t="inlineStr">
+      <c r="R21" s="14" t="n"/>
+      <c r="S21" s="14" t="n"/>
+      <c r="T21" s="14" t="n"/>
+      <c r="U21" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" (бледно-розовый, one size)</t>
         </is>
       </c>
-      <c r="V21" s="4" t="n"/>
-      <c r="W21" s="4" t="n"/>
-      <c r="X21" s="4" t="n"/>
-      <c r="Y21" s="4" t="inlineStr">
-        <is>
-          <t>Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
-        </is>
-      </c>
-      <c r="Z21" s="4" t="n"/>
-      <c r="AA21" s="4" t="n"/>
-      <c r="AB21" s="4" t="n"/>
+      <c r="V21" s="14" t="n"/>
+      <c r="W21" s="14" t="n"/>
+      <c r="X21" s="14" t="n"/>
+      <c r="Y21" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
+        </is>
+      </c>
+      <c r="Z21" s="14" t="n"/>
+      <c r="AA21" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB21" s="14" t="n"/>
     </row>
     <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" - Розовый барби</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Розовый барби</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="7" t="n">
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="14" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="L22" s="7" t="n">
+      <c r="L22" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M22" s="14" t="inlineStr">
         <is>
           <t>2023-04-12</t>
         </is>
       </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="N22" s="14" t="inlineStr">
         <is>
           <t>2023-04-12</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="O22" s="14" t="inlineStr">
         <is>
           <t>Оплачен 1</t>
         </is>
       </c>
-      <c r="P22" s="4" t="inlineStr">
+      <c r="P22" s="14" t="inlineStr">
         <is>
           <t>6295</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
+      <c r="Q22" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R22" s="4" t="n"/>
-      <c r="S22" s="4" t="n"/>
-      <c r="T22" s="4" t="n"/>
-      <c r="U22" s="4" t="inlineStr">
+      <c r="R22" s="14" t="n"/>
+      <c r="S22" s="14" t="n"/>
+      <c r="T22" s="14" t="n"/>
+      <c r="U22" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream"</t>
         </is>
       </c>
-      <c r="V22" s="4" t="n"/>
-      <c r="W22" s="4" t="n"/>
-      <c r="X22" s="4" t="n"/>
-      <c r="Y22" s="4" t="inlineStr">
-        <is>
-          <t>Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z22" s="4" t="inlineStr">
+      <c r="V22" s="14" t="n"/>
+      <c r="W22" s="14" t="n"/>
+      <c r="X22" s="14" t="n"/>
+      <c r="Y22" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z22" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream"; Воротничок "Dream" (белый, one size); Воротничок "Dream" (бледно-розовый, one size); Воротничок "Dream" (лавандовый, one size); Воротничок "Dream" (мятный, one size)</t>
         </is>
       </c>
-      <c r="AA22" s="4" t="n"/>
-      <c r="AB22" s="4" t="n"/>
+      <c r="AA22" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB22" s="14" t="n"/>
     </row>
     <row r="23" ht="48" customHeight="1">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Боди с длинным рукавом "На моих условиях"</t>
         </is>
       </c>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>100002</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="14" t="inlineStr">
         <is>
           <t>Для склейки не использовал: в старых заказах в артикул часто попадала цена.</t>
         </is>
       </c>
-      <c r="H23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" s="7" t="n">
+      <c r="H23" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="17" t="n">
         <v>25657.14</v>
       </c>
-      <c r="L23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="L23" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="14" t="inlineStr">
         <is>
           <t>2026-04-04</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="N23" s="14" t="inlineStr">
         <is>
           <t>2026-04-04</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr">
+      <c r="O23" s="14" t="inlineStr">
         <is>
           <t>Ошибка оплаты 1</t>
         </is>
       </c>
-      <c r="P23" s="4" t="inlineStr">
+      <c r="P23" s="14" t="inlineStr">
         <is>
           <t>237513</t>
         </is>
       </c>
-      <c r="Q23" s="4" t="inlineStr">
+      <c r="Q23" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R23" s="8" t="inlineStr">
+      <c r="R23" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/bodi-s-dlinnym-rukavom-na-moih-usloviyah-2/</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr">
+      <c r="S23" s="14" t="inlineStr">
         <is>
           <t>Бестселлеры, Боди и топы, Всё по плечу, Все товары</t>
         </is>
       </c>
-      <c r="T23" s="4" t="n"/>
-      <c r="U23" s="4" t="inlineStr">
+      <c r="T23" s="14" t="n"/>
+      <c r="U23" s="14" t="inlineStr">
         <is>
           <t>Боди с длинным рукавом "На моих условиях"</t>
         </is>
       </c>
-      <c r="V23" s="4" t="n"/>
-      <c r="W23" s="4" t="n"/>
-      <c r="X23" s="4" t="n"/>
-      <c r="Y23" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
-        </is>
-      </c>
-      <c r="Z23" s="4" t="inlineStr">
+      <c r="V23" s="14" t="n"/>
+      <c r="W23" s="14" t="n"/>
+      <c r="X23" s="14" t="n"/>
+      <c r="Y23" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
+        </is>
+      </c>
+      <c r="Z23" s="14" t="inlineStr">
         <is>
           <t>Боди с длинным рукавом "На моих условиях" (тёмно-синий); Боди с длинным рукавом "На моих условиях" (тёмно-синий) (M); Боди с длинным рукавом "На моих условиях" (тёмно-синий) (S); Боди с длинным рукавом "На моих условиях" (молочный); Боди с длинным рукавом "На моих условиях" (молочный) (M); Боди с длинным рукавом "На моих условиях" (молочный) (S)</t>
         </is>
       </c>
-      <c r="AA23" s="4" t="n"/>
-      <c r="AB23" s="4" t="n"/>
+      <c r="AA23" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB23" s="14" t="n"/>
     </row>
     <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>Кардиган 2MY x Maria Kalashnikova - терракотовый, XS</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>терракотовый</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>28000</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>Похоже на цену, а не на артикул. Для поиска карточки не использовал.</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K24" s="7" t="n">
+      <c r="H24" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="17" t="n">
         <v>24900</v>
       </c>
-      <c r="L24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="L24" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="14" t="inlineStr">
         <is>
           <t>2025-01-18</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="N24" s="14" t="inlineStr">
         <is>
           <t>2025-01-18</t>
         </is>
       </c>
-      <c r="O24" s="4" t="inlineStr">
+      <c r="O24" s="14" t="inlineStr">
         <is>
           <t>Отменён 1</t>
         </is>
       </c>
-      <c r="P24" s="4" t="inlineStr">
+      <c r="P24" s="14" t="inlineStr">
         <is>
           <t>66735</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="inlineStr">
+      <c r="Q24" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R24" s="8" t="inlineStr">
+      <c r="R24" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/kardigan-2my-x-maria-kalashnikova/</t>
         </is>
       </c>
-      <c r="S24" s="4" t="inlineStr">
+      <c r="S24" s="14" t="inlineStr">
         <is>
           <t>Все товары</t>
         </is>
       </c>
-      <c r="T24" s="4" t="inlineStr">
+      <c r="T24" s="14" t="inlineStr">
         <is>
           <t>предзаказ</t>
         </is>
       </c>
-      <c r="U24" s="4" t="inlineStr">
+      <c r="U24" s="14" t="inlineStr">
         <is>
           <t>Кардиган 2MY x Maria Kalashnikova</t>
         </is>
       </c>
-      <c r="V24" s="4" t="n"/>
-      <c r="W24" s="4" t="n"/>
-      <c r="X24" s="4" t="n"/>
-      <c r="Y24" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z24" s="4" t="inlineStr">
+      <c r="V24" s="14" t="n"/>
+      <c r="W24" s="14" t="n"/>
+      <c r="X24" s="14" t="n"/>
+      <c r="Y24" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z24" s="14" t="inlineStr">
         <is>
           <t>Кардиган 2MY x Maria Kalashnikova; Кардиган 2MY x Maria Kalashnikova (Молочный, S-M); Кардиган 2MY x Maria Kalashnikova (Молочный, XS); Кардиган 2MY x Maria Kalashnikova (XS, Шоколадный); Кардиган 2MY x Maria Kalashnikova (S-M, Шоколадный)</t>
         </is>
       </c>
-      <c r="AA24" s="4" t="n"/>
-      <c r="AB24" s="4" t="n"/>
+      <c r="AA24" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB24" s="14" t="n"/>
     </row>
     <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>Топ сатиновый "Крем-сода" - Кремовый, XS</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Кремовый</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>96000</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>Похоже на цену, а не на артикул. Для поиска карточки не использовал.</t>
         </is>
       </c>
-      <c r="H25" s="6" t="n">
+      <c r="H25" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="6" t="n">
+      <c r="I25" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="K25" s="7" t="n">
+      <c r="K25" s="17" t="n">
         <v>23700</v>
       </c>
-      <c r="L25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="L25" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="14" t="inlineStr">
         <is>
           <t>2025-07-09</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="N25" s="14" t="inlineStr">
         <is>
           <t>2025-07-10</t>
         </is>
       </c>
-      <c r="O25" s="4" t="inlineStr">
+      <c r="O25" s="14" t="inlineStr">
         <is>
           <t>Отменён 3</t>
         </is>
       </c>
-      <c r="P25" s="4" t="inlineStr">
+      <c r="P25" s="14" t="inlineStr">
         <is>
           <t>214539, 214580, 214647</t>
         </is>
       </c>
-      <c r="Q25" s="4" t="inlineStr">
+      <c r="Q25" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R25" s="8" t="inlineStr">
+      <c r="R25" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/top-satinovyj-krem-soda/</t>
         </is>
       </c>
-      <c r="S25" s="4" t="inlineStr">
+      <c r="S25" s="14" t="inlineStr">
         <is>
           <t>Боди и топы, Все товары, Замедляя шаг, Костюмы, Лето</t>
         </is>
       </c>
-      <c r="T25" s="4" t="n"/>
-      <c r="U25" s="4" t="inlineStr">
+      <c r="T25" s="14" t="n"/>
+      <c r="U25" s="14" t="inlineStr">
         <is>
           <t>Топ сатиновый "Крем-сода"</t>
         </is>
       </c>
-      <c r="V25" s="4" t="n"/>
-      <c r="W25" s="4" t="n"/>
-      <c r="X25" s="4" t="n"/>
-      <c r="Y25" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Та же модель и цвет на складе есть, этого размера нет. Ниже карточки, которые уже заведены.</t>
-        </is>
-      </c>
-      <c r="Z25" s="4" t="inlineStr">
+      <c r="V25" s="14" t="n"/>
+      <c r="W25" s="14" t="n"/>
+      <c r="X25" s="14" t="n"/>
+      <c r="Y25" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Та же модель и цвет на складе есть, этого размера нет. Ниже карточки, которые уже заведены.</t>
+        </is>
+      </c>
+      <c r="Z25" s="14" t="inlineStr">
         <is>
           <t>Топ сатиновый "Крем-сода" (Кремовый, S-M)</t>
         </is>
       </c>
-      <c r="AA25" s="4" t="n"/>
-      <c r="AB25" s="4" t="n"/>
+      <c r="AA25" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB25" s="14" t="n"/>
     </row>
     <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>Лонгслив из мохера "Прочная связь" - S</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>100043</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>Для склейки не использовал: в старых заказах в артикул часто попадала цена.</t>
         </is>
       </c>
-      <c r="H26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" s="7" t="n">
+      <c r="H26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="17" t="n">
         <v>22761.9</v>
       </c>
-      <c r="L26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="L26" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="14" t="inlineStr">
         <is>
           <t>2026-01-17</t>
         </is>
       </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="N26" s="14" t="inlineStr">
         <is>
           <t>2026-01-17</t>
         </is>
       </c>
-      <c r="O26" s="4" t="inlineStr">
+      <c r="O26" s="14" t="inlineStr">
         <is>
           <t>Ошибка оплаты 1</t>
         </is>
       </c>
-      <c r="P26" s="4" t="inlineStr">
+      <c r="P26" s="14" t="inlineStr">
         <is>
           <t>00252</t>
         </is>
       </c>
-      <c r="Q26" s="4" t="inlineStr">
+      <c r="Q26" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R26" s="8" t="inlineStr">
+      <c r="R26" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/longsliv-iz-mohera-prochnaya-svyaz-siyanie/</t>
         </is>
       </c>
-      <c r="S26" s="4" t="inlineStr">
+      <c r="S26" s="14" t="inlineStr">
         <is>
           <t>Все товары, Ночь перед Рождеством</t>
         </is>
       </c>
-      <c r="T26" s="4" t="n"/>
-      <c r="U26" s="4" t="n"/>
-      <c r="V26" s="4" t="n"/>
-      <c r="W26" s="4" t="n"/>
-      <c r="X26" s="4" t="n"/>
-      <c r="Y26" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
-        </is>
-      </c>
-      <c r="Z26" s="4" t="inlineStr">
-        <is>
-          <t>Лонгслив из мохера "Прочная связь" (розовый) (S); Лонгслив из мохера "Прочная связь", Молочный (S); Лонгслив из мохера "Прочная связь", Серый (S)</t>
-        </is>
-      </c>
-      <c r="AA26" s="4" t="n"/>
-      <c r="AB26" s="4" t="n"/>
+      <c r="T26" s="14" t="n"/>
+      <c r="U26" s="14" t="inlineStr">
+        <is>
+          <t>Лонгслив из мохера "Прочная связь" (сияние) (S)</t>
+        </is>
+      </c>
+      <c r="V26" s="14" t="n"/>
+      <c r="W26" s="14" t="inlineStr">
+        <is>
+          <t>Лонгсливы и свитеры</t>
+        </is>
+      </c>
+      <c r="X26" s="14" t="inlineStr">
+        <is>
+          <t>в архиве</t>
+        </is>
+      </c>
+      <c r="Y26" s="14" t="inlineStr">
+        <is>
+          <t>В заказе стоит ссылка на эту карточку. Она в архиве, поэтому в прошлый список не попала. Подтверждено 8 октября 2026.</t>
+        </is>
+      </c>
+      <c r="Z26" s="14" t="inlineStr">
+        <is>
+          <t>Рядом есть живые карточки размера S: розовый, молочный, серый. У этого заказа ссылка именно на сияние.</t>
+        </is>
+      </c>
+      <c r="AA26" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB26" s="14" t="n"/>
     </row>
     <row r="27" ht="48" customHeight="1">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>Платье с вырезом на спине серое</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>серое</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K27" s="7" t="n">
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="14" t="n"/>
+      <c r="G27" s="14" t="n"/>
+      <c r="H27" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" s="17" t="n">
         <v>14400</v>
       </c>
-      <c r="L27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="L27" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="14" t="inlineStr">
         <is>
           <t>2023-08-11</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="N27" s="14" t="inlineStr">
         <is>
           <t>2023-08-11</t>
         </is>
       </c>
-      <c r="O27" s="4" t="inlineStr">
+      <c r="O27" s="14" t="inlineStr">
         <is>
           <t>Отменён 1</t>
         </is>
       </c>
-      <c r="P27" s="4" t="inlineStr">
+      <c r="P27" s="14" t="inlineStr">
         <is>
           <t>7006</t>
         </is>
       </c>
-      <c r="Q27" s="4" t="inlineStr">
+      <c r="Q27" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R27" s="4" t="n"/>
-      <c r="S27" s="4" t="n"/>
-      <c r="T27" s="4" t="n"/>
-      <c r="U27" s="4" t="inlineStr">
+      <c r="R27" s="14" t="n"/>
+      <c r="S27" s="14" t="n"/>
+      <c r="T27" s="14" t="n"/>
+      <c r="U27" s="14" t="inlineStr">
         <is>
           <t>Платье с вырезом на спине (серый, one size)</t>
         </is>
       </c>
-      <c r="V27" s="4" t="n"/>
-      <c r="W27" s="4" t="n"/>
-      <c r="X27" s="4" t="n"/>
-      <c r="Y27" s="4" t="inlineStr">
-        <is>
-          <t>Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
-        </is>
-      </c>
-      <c r="Z27" s="4" t="n"/>
-      <c r="AA27" s="4" t="n"/>
-      <c r="AB27" s="4" t="n"/>
+      <c r="V27" s="14" t="n"/>
+      <c r="W27" s="14" t="n"/>
+      <c r="X27" s="14" t="n"/>
+      <c r="Y27" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
+        </is>
+      </c>
+      <c r="Z27" s="14" t="n"/>
+      <c r="AA27" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB27" s="14" t="n"/>
     </row>
     <row r="28" ht="48" customHeight="1">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" - Неоновый</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Неоновый</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="6" t="n">
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="14" t="n"/>
+      <c r="G28" s="14" t="n"/>
+      <c r="H28" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I28" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="6" t="n">
+      <c r="I28" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="K28" s="7" t="n">
+      <c r="K28" s="17" t="n">
         <v>11400</v>
       </c>
-      <c r="L28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="4" t="inlineStr">
+      <c r="L28" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="14" t="inlineStr">
         <is>
           <t>2022-05-12</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="N28" s="14" t="inlineStr">
         <is>
           <t>2022-05-16</t>
         </is>
       </c>
-      <c r="O28" s="4" t="inlineStr">
+      <c r="O28" s="14" t="inlineStr">
         <is>
           <t>Отменён 3</t>
         </is>
       </c>
-      <c r="P28" s="4" t="inlineStr">
+      <c r="P28" s="14" t="inlineStr">
         <is>
           <t>5289, 5290, 5292</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr">
+      <c r="Q28" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R28" s="4" t="n"/>
-      <c r="S28" s="4" t="n"/>
-      <c r="T28" s="4" t="n"/>
-      <c r="U28" s="4" t="inlineStr">
+      <c r="R28" s="14" t="n"/>
+      <c r="S28" s="14" t="n"/>
+      <c r="T28" s="14" t="n"/>
+      <c r="U28" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream"</t>
         </is>
       </c>
-      <c r="V28" s="4" t="n"/>
-      <c r="W28" s="4" t="n"/>
-      <c r="X28" s="4" t="n"/>
-      <c r="Y28" s="4" t="inlineStr">
-        <is>
-          <t>Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z28" s="4" t="inlineStr">
+      <c r="V28" s="14" t="n"/>
+      <c r="W28" s="14" t="n"/>
+      <c r="X28" s="14" t="n"/>
+      <c r="Y28" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z28" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream"; Воротничок "Dream" (белый, one size); Воротничок "Dream" (бледно-розовый, one size); Воротничок "Dream" (лавандовый, one size); Воротничок "Dream" (мятный, one size)</t>
         </is>
       </c>
-      <c r="AA28" s="4" t="n"/>
-      <c r="AB28" s="4" t="n"/>
+      <c r="AA28" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB28" s="14" t="n"/>
     </row>
     <row r="29" ht="48" customHeight="1">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Чепчик "Звездное небо" - Серый</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Серый</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>18000</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Похоже на цену, а не на артикул. Для поиска карточки не использовал.</t>
         </is>
       </c>
-      <c r="H29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" s="7" t="n">
+      <c r="H29" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="17" t="n">
         <v>8900</v>
       </c>
-      <c r="L29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="L29" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="14" t="inlineStr">
         <is>
           <t>2025-01-07</t>
         </is>
       </c>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="N29" s="14" t="inlineStr">
         <is>
           <t>2025-01-07</t>
         </is>
       </c>
-      <c r="O29" s="4" t="inlineStr">
+      <c r="O29" s="14" t="inlineStr">
         <is>
           <t>Отменён 1</t>
         </is>
       </c>
-      <c r="P29" s="4" t="inlineStr">
+      <c r="P29" s="14" t="inlineStr">
         <is>
           <t>49168</t>
         </is>
       </c>
-      <c r="Q29" s="4" t="inlineStr">
+      <c r="Q29" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R29" s="8" t="inlineStr">
+      <c r="R29" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/sample/chepchik-zvezdnoe-nebo/</t>
         </is>
       </c>
-      <c r="S29" s="4" t="inlineStr">
+      <c r="S29" s="14" t="inlineStr">
         <is>
           <t>Sample</t>
         </is>
       </c>
-      <c r="T29" s="4" t="n"/>
-      <c r="U29" s="4" t="inlineStr">
+      <c r="T29" s="14" t="n"/>
+      <c r="U29" s="14" t="inlineStr">
         <is>
           <t>Чепчик "Звездное небо"</t>
         </is>
       </c>
-      <c r="V29" s="4" t="n"/>
-      <c r="W29" s="4" t="n"/>
-      <c r="X29" s="4" t="n"/>
-      <c r="Y29" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z29" s="4" t="inlineStr">
+      <c r="V29" s="14" t="n"/>
+      <c r="W29" s="14" t="n"/>
+      <c r="X29" s="14" t="n"/>
+      <c r="Y29" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z29" s="14" t="inlineStr">
         <is>
           <t>Чепчик "Звездное небо"; Чепчик "Звездное небо" (белый, one size)</t>
         </is>
       </c>
-      <c r="AA29" s="4" t="n"/>
-      <c r="AB29" s="4" t="n"/>
+      <c r="AA29" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB29" s="14" t="n"/>
     </row>
     <row r="30" ht="48" customHeight="1">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>Топ "Touch" - Белый</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>Белый</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" s="7" t="n">
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="14" t="n"/>
+      <c r="G30" s="14" t="n"/>
+      <c r="H30" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="17" t="n">
         <v>3900</v>
       </c>
-      <c r="L30" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="L30" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="14" t="inlineStr">
         <is>
           <t>2023-05-11</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="N30" s="14" t="inlineStr">
         <is>
           <t>2023-05-11</t>
         </is>
       </c>
-      <c r="O30" s="4" t="inlineStr">
+      <c r="O30" s="14" t="inlineStr">
         <is>
           <t>Отменён 1</t>
         </is>
       </c>
-      <c r="P30" s="4" t="inlineStr">
+      <c r="P30" s="14" t="inlineStr">
         <is>
           <t>6500</t>
         </is>
       </c>
-      <c r="Q30" s="4" t="inlineStr">
+      <c r="Q30" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R30" s="4" t="n"/>
-      <c r="S30" s="4" t="n"/>
-      <c r="T30" s="4" t="n"/>
-      <c r="U30" s="4" t="inlineStr">
+      <c r="R30" s="14" t="n"/>
+      <c r="S30" s="14" t="n"/>
+      <c r="T30" s="14" t="n"/>
+      <c r="U30" s="14" t="inlineStr">
         <is>
           <t>Топ "Touch"</t>
         </is>
       </c>
-      <c r="V30" s="4" t="n"/>
-      <c r="W30" s="4" t="n"/>
-      <c r="X30" s="4" t="n"/>
-      <c r="Y30" s="4" t="inlineStr">
-        <is>
-          <t>Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
-        </is>
-      </c>
-      <c r="Z30" s="4" t="inlineStr">
+      <c r="V30" s="14" t="n"/>
+      <c r="W30" s="14" t="n"/>
+      <c r="X30" s="14" t="n"/>
+      <c r="Y30" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Та же модель на складе есть, этого цвета нет. Если цвета правда нет, добавьте отдельно. Если это одна из карточек ниже, напишите её в решении.</t>
+        </is>
+      </c>
+      <c r="Z30" s="14" t="inlineStr">
         <is>
           <t>Топ "Touch"; Топ "Touch" (кремовый, one size)</t>
         </is>
       </c>
-      <c r="AA30" s="4" t="n"/>
-      <c r="AB30" s="4" t="n"/>
+      <c r="AA30" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB30" s="14" t="n"/>
     </row>
     <row r="31" ht="48" customHeight="1">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" - Лавандовый</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>Лавандовый</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I31" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="14" t="inlineStr">
         <is>
           <t>2022-08-24</t>
         </is>
       </c>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="N31" s="14" t="inlineStr">
         <is>
           <t>2022-08-24</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr">
+      <c r="O31" s="14" t="inlineStr">
         <is>
           <t>Отменён 1</t>
         </is>
       </c>
-      <c r="P31" s="4" t="inlineStr">
+      <c r="P31" s="14" t="inlineStr">
         <is>
           <t>5407</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
+      <c r="Q31" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R31" s="4" t="n"/>
-      <c r="S31" s="4" t="n"/>
-      <c r="T31" s="4" t="n"/>
-      <c r="U31" s="4" t="inlineStr">
+      <c r="R31" s="14" t="n"/>
+      <c r="S31" s="14" t="n"/>
+      <c r="T31" s="14" t="n"/>
+      <c r="U31" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" (лавандовый, one size)</t>
         </is>
       </c>
-      <c r="V31" s="4" t="n"/>
-      <c r="W31" s="4" t="n"/>
-      <c r="X31" s="4" t="n"/>
-      <c r="Y31" s="4" t="inlineStr">
-        <is>
-          <t>Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
-        </is>
-      </c>
-      <c r="Z31" s="4" t="n"/>
-      <c r="AA31" s="4" t="n"/>
-      <c r="AB31" s="4" t="n"/>
+      <c r="V31" s="14" t="n"/>
+      <c r="W31" s="14" t="n"/>
+      <c r="X31" s="14" t="n"/>
+      <c r="Y31" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
+        </is>
+      </c>
+      <c r="Z31" s="14" t="n"/>
+      <c r="AA31" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB31" s="14" t="n"/>
     </row>
     <row r="32" ht="48" customHeight="1">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" - Мятный</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>Мятный</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I32" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K32" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="14" t="inlineStr">
         <is>
           <t>2022-08-16</t>
         </is>
       </c>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="N32" s="14" t="inlineStr">
         <is>
           <t>2022-08-16</t>
         </is>
       </c>
-      <c r="O32" s="4" t="inlineStr">
+      <c r="O32" s="14" t="inlineStr">
         <is>
           <t>Отменён 1</t>
         </is>
       </c>
-      <c r="P32" s="4" t="inlineStr">
+      <c r="P32" s="14" t="inlineStr">
         <is>
           <t>5396</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr">
+      <c r="Q32" s="14" t="inlineStr">
         <is>
           <t>Карточка товара на сайте уже удалена, осталось название в заказе</t>
         </is>
       </c>
-      <c r="R32" s="4" t="n"/>
-      <c r="S32" s="4" t="n"/>
-      <c r="T32" s="4" t="n"/>
-      <c r="U32" s="4" t="inlineStr">
+      <c r="R32" s="14" t="n"/>
+      <c r="S32" s="14" t="n"/>
+      <c r="T32" s="14" t="n"/>
+      <c r="U32" s="14" t="inlineStr">
         <is>
           <t>Воротничок "Dream" (мятный, one size)</t>
         </is>
       </c>
-      <c r="V32" s="4" t="n"/>
-      <c r="W32" s="4" t="n"/>
-      <c r="X32" s="4" t="n"/>
-      <c r="Y32" s="4" t="inlineStr">
-        <is>
-          <t>Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
-        </is>
-      </c>
-      <c r="Z32" s="4" t="n"/>
-      <c r="AA32" s="4" t="n"/>
-      <c r="AB32" s="4" t="n"/>
+      <c r="V32" s="14" t="n"/>
+      <c r="W32" s="14" t="n"/>
+      <c r="X32" s="14" t="n"/>
+      <c r="Y32" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Совпали модель и цвет. Размер в заказе не указан, на складе карточка одна.</t>
+        </is>
+      </c>
+      <c r="Z32" s="14" t="n"/>
+      <c r="AA32" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB32" s="14" t="n"/>
     </row>
     <row r="33" ht="48" customHeight="1">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Похоже на существующий, подтвердите</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>Существующий товар</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
         <is>
           <t>Подстаканник вязаный (подарок)</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>00484</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="14" t="inlineStr">
         <is>
           <t>Для склейки не использовал: в старых заказах в артикул часто попадала цена.</t>
         </is>
       </c>
-      <c r="H33" s="6" t="n">
+      <c r="H33" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="I33" s="6" t="n">
+      <c r="I33" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="J33" s="6" t="n">
+      <c r="J33" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="K33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" s="4" t="inlineStr">
+      <c r="K33" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="14" t="inlineStr">
         <is>
           <t>2024-11-01</t>
         </is>
       </c>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="N33" s="14" t="inlineStr">
         <is>
           <t>2025-06-26</t>
         </is>
       </c>
-      <c r="O33" s="4" t="inlineStr">
+      <c r="O33" s="14" t="inlineStr">
         <is>
           <t>Отменён 2, В обработке 2, Оплачен 1</t>
         </is>
       </c>
-      <c r="P33" s="4" t="inlineStr">
+      <c r="P33" s="14" t="inlineStr">
         <is>
           <t>13625, 66816, 167734, 206029, 206109</t>
         </is>
       </c>
-      <c r="Q33" s="4" t="inlineStr">
+      <c r="Q33" s="14" t="inlineStr">
         <is>
           <t>Карточка на сайте открывается</t>
         </is>
       </c>
-      <c r="R33" s="8" t="inlineStr">
+      <c r="R33" s="18" t="inlineStr">
         <is>
           <t>https://2mymoods.ru/shop/all/podstakannik-vyazanyj-podarok/</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr">
+      <c r="S33" s="14" t="inlineStr">
         <is>
           <t>Все товары</t>
         </is>
       </c>
-      <c r="T33" s="4" t="n"/>
-      <c r="U33" s="4" t="inlineStr">
+      <c r="T33" s="14" t="n"/>
+      <c r="U33" s="14" t="inlineStr">
         <is>
           <t>Подстаканник вязаный</t>
         </is>
       </c>
-      <c r="V33" s="4" t="n"/>
-      <c r="W33" s="4" t="n"/>
-      <c r="X33" s="4" t="n"/>
-      <c r="Y33" s="4" t="inlineStr">
-        <is>
-          <t>Прежняя ссылка на склад больше не открывается. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
-        </is>
-      </c>
-      <c r="Z33" s="4" t="inlineStr">
+      <c r="V33" s="14" t="n"/>
+      <c r="W33" s="14" t="n"/>
+      <c r="X33" s="14" t="n"/>
+      <c r="Y33" s="14" t="inlineStr">
+        <is>
+          <t>Подтверждено 8 октября 2026: это эта карточка. Прежняя ссылка на склад больше не открывается. Похожих карточек несколько, одну я не выбрал. Если это одна из них, впишите название в решение. Если нет, оставьте как новый товар.</t>
+        </is>
+      </c>
+      <c r="Z33" s="14" t="inlineStr">
         <is>
           <t>Подстаканник вязаный; Подстаканник вязаный (one size, Микс)</t>
         </is>
       </c>
-      <c r="AA33" s="4" t="n"/>
-      <c r="AB33" s="4" t="n"/>
+      <c r="AA33" s="14" t="inlineStr">
+        <is>
+          <t>верно</t>
+        </is>
+      </c>
+      <c r="AB33" s="14" t="n"/>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="9" t="n">

</xml_diff>